<commit_message>
data: Week 17 AMS data - Tonor, White Mulberry + processed CSVs
</commit_message>
<xml_diff>
--- a/data/ams_weekly_data/Tonor/ads_report_week17.xlsx
+++ b/data/ams_weekly_data/Tonor/ads_report_week17.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Week 17\Week 17\ams_weekly_data\Tonor\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Other computers\My Laptop\D\Nitesh\Weekly Report - B2B + B2C\FastAPI\data\ams_weekly_data\Tonor\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBF8FA5F-68CC-4665-81D5-5F13738EEBDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="2" xr2:uid="{C2EB3544-0B30-4B5A-9817-98DE85FBF6BC}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{C2EB3544-0B30-4B5A-9817-98DE85FBF6BC}"/>
   </bookViews>
   <sheets>
     <sheet name="SP" sheetId="1" r:id="rId1"/>

</xml_diff>